<commit_message>
Fix récap 18h + email iryannhassim + Excel
</commit_message>
<xml_diff>
--- a/suivi_stages.xlsx
+++ b/suivi_stages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iryan\Documents\GitHub\job-alert\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF1F2BDE-DFC5-44C5-B795-F5EFAACC2561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7404DF-EF5C-43FF-91E1-1F6ED8431C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22276" windowHeight="13276" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22276" windowHeight="13276" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suivi des candidatures" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="113">
   <si>
     <t>🎓 SUIVI DES CANDIDATURES DE STAGE</t>
   </si>
@@ -340,6 +340,27 @@
   </si>
   <si>
     <t>Partout sauf que s'il n'est pas en île de France, il doit être prestigieux</t>
+  </si>
+  <si>
+    <t>https://www.rothschildandco.com/en/careers/students-and-graduates/opportunities/</t>
+  </si>
+  <si>
+    <t>Rothschild &amp; Co</t>
+  </si>
+  <si>
+    <t>Tout poste lié à l'ESG</t>
+  </si>
+  <si>
+    <t>Edmond de Rothschild</t>
+  </si>
+  <si>
+    <t>https://evht.fa.ocs.oraclecloud.eu/hcmUI/CandidateExperience/fr/sites/CX_7001/jobs?mode=location</t>
+  </si>
+  <si>
+    <t>Le poste de stagiaire ou alternant peut être partout dans le monde ou je n'ai pas besoin d'être sponsorisé (exemple : suisse, Espagne...)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Théophile </t>
   </si>
 </sst>
 </file>
@@ -1828,20 +1849,42 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="32"/>
-      <c r="B23" s="46"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="35"/>
+      <c r="A23" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="B23" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="32" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" s="35" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="24" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="32"/>
-      <c r="B24" s="32"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="42"/>
+      <c r="B24" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="32" t="s">
+        <v>111</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" s="42" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="32"/>

</xml_diff>